<commit_message>
A count scales from units, not from the file's currency scale
Money and a count start from different places, so they cannot divide the same
way. Money is stated against the file's own unit: a file in US$m carrying a
line declared US$m divides by one, and one declared US$bn by a thousand. A
count has no such base — 162,369 customers is 162,369 units — so a count
declared in millions divides by a million and prints as 0.16mn.

A count is also named the way a pack writes it, with no currency in front:
"mn", not "m" and not "US$m". And a figure scaled below one keeps two
decimals rather than rounding itself away, so 0.16 does not read as 0.2.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4DDZgm6WRNJpLjFRThM8B
</commit_message>
<xml_diff>
--- a/iwpb-sg-dashboard/sample/IWPB_unit_and_rollup_sample.xlsx
+++ b/iwpb-sg-dashboard/sample/IWPB_unit_and_rollup_sample.xlsx
@@ -450,7 +450,7 @@
     <col min="1" max="1" width="48.83203125" customWidth="1"/>
     <col min="2" max="2" width="33.83203125" customWidth="1"/>
     <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="45.83203125" customWidth="1"/>
+    <col min="4" max="4" width="46.83203125" customWidth="1"/>
     <col min="5" max="5" width="11.83203125" customWidth="1"/>
     <col min="6" max="6" width="17.83203125" customWidth="1"/>
     <col min="7" max="7" width="11.83203125" customWidth="1"/>
@@ -773,7 +773,7 @@
         <v>number</v>
       </c>
       <c r="E15" s="2" t="str">
-        <v>m</v>
+        <v>mn</v>
       </c>
       <c r="F15" s="5">
         <v>162369</v>
@@ -973,7 +973,7 @@
         <v>no total</v>
       </c>
       <c r="D26" s="2" t="str">
-        <v>%, number, m, US$m are never added together</v>
+        <v>%, number, mn, US$m are never added together</v>
       </c>
     </row>
     <row r="28">

</xml_diff>